<commit_message>
Add analysis artifacts and updated performance workbook
</commit_message>
<xml_diff>
--- a/job_scheduler/data/all_model_data_by_rank.xlsx
+++ b/job_scheduler/data/all_model_data_by_rank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/imtiazevan/Desktop/Projects/temp/MPR_System_Beta/job_scheduler/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FFE38C-DEDB-E747-B3CE-092BC4C298A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F342CEA1-3B50-994B-8FFE-351B0B4B1026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16300" activeTab="3" xr2:uid="{15444B7F-6FA5-5E4D-9AAE-4CEB8B7D2F02}"/>
+    <workbookView xWindow="3400" yWindow="500" windowWidth="28800" windowHeight="16300" activeTab="3" xr2:uid="{15444B7F-6FA5-5E4D-9AAE-4CEB8B7D2F02}"/>
   </bookViews>
   <sheets>
     <sheet name="comd" sheetId="16" r:id="rId1"/>
@@ -2140,29 +2140,29 @@
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f t="shared" ref="A2:A15" si="0">B2/$B$16</f>
-        <v>0.54614207182740815</v>
+        <v>0.5853651583847439</v>
       </c>
       <c r="B2">
-        <v>78.388528140000005</v>
+        <v>80.023503000000005</v>
       </c>
       <c r="C2">
-        <v>46.957853450000002</v>
+        <v>53.109729000000002</v>
       </c>
       <c r="D2">
-        <f t="shared" ref="D2:D15" si="1">1/C2*100</f>
-        <v>2.1295692339616519</v>
+        <f t="shared" ref="D2:D31" si="1">1/C2*100</f>
+        <v>1.8828941868635782</v>
       </c>
       <c r="E2">
         <f t="shared" ref="E2:E15" si="2">D2-$D$16</f>
-        <v>1.1295692339616519</v>
+        <v>0.88289418686357823</v>
       </c>
       <c r="F2">
         <f>IFERROR(E2/G2,0)</f>
-        <v>2.4888167945192365</v>
+        <v>2.1293294683682777</v>
       </c>
       <c r="G2">
         <f>$A$16-A2</f>
-        <v>0.45385792817259185</v>
+        <v>0.4146348416152561</v>
       </c>
       <c r="H2">
         <v>1000</v>
@@ -2171,29 +2171,29 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>0.54894550711202528</v>
+        <v>0.60720817620285383</v>
       </c>
       <c r="B3">
-        <v>78.79090909</v>
+        <v>83.009596000000002</v>
       </c>
       <c r="C3">
-        <v>51.545171330000002</v>
+        <v>60.344082</v>
       </c>
       <c r="D3">
         <f t="shared" si="1"/>
-        <v>1.9400459329116369</v>
+        <v>1.6571633321060382</v>
       </c>
       <c r="E3">
         <f t="shared" si="2"/>
-        <v>0.94004593291163685</v>
+        <v>0.65716333210603817</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F16" si="3">IFERROR(E3/G3,0)</f>
-        <v>2.0841072370054179</v>
+        <v>1.6730575645724854</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G16" si="4">$A$16-A3</f>
-        <v>0.45105449288797472</v>
+        <v>0.39279182379714617</v>
       </c>
       <c r="H3">
         <v>1100</v>
@@ -2202,29 +2202,29 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>0.60564554719726515</v>
+        <v>0.61983106495366957</v>
       </c>
       <c r="B4">
-        <v>86.929144390000005</v>
+        <v>84.735232999999994</v>
       </c>
       <c r="C4">
-        <v>57.11660741</v>
+        <v>62.392927</v>
       </c>
       <c r="D4">
         <f t="shared" si="1"/>
-        <v>1.7508042675253843</v>
+        <v>1.6027457727700449</v>
       </c>
       <c r="E4">
         <f t="shared" si="2"/>
-        <v>0.75080426752538432</v>
+        <v>0.60274577277004493</v>
       </c>
       <c r="F4">
         <f t="shared" si="3"/>
-        <v>1.9038818052878785</v>
+        <v>1.5854682411033652</v>
       </c>
       <c r="G4">
         <f t="shared" si="4"/>
-        <v>0.39435445280273485</v>
+        <v>0.38016893504633043</v>
       </c>
       <c r="H4">
         <v>1200</v>
@@ -2233,29 +2233,29 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>0.63098893214681462</v>
+        <v>0.64065019942654</v>
       </c>
       <c r="B5">
-        <v>90.566715540000004</v>
+        <v>87.581354000000005</v>
       </c>
       <c r="C5">
-        <v>64.170137850000003</v>
+        <v>66.772675000000007</v>
       </c>
       <c r="D5">
         <f t="shared" si="1"/>
-        <v>1.5583572569807094</v>
+        <v>1.4976185992249074</v>
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>0.55835725698070937</v>
+        <v>0.49761859922490737</v>
       </c>
       <c r="F5">
         <f t="shared" si="3"/>
-        <v>1.5131179133165111</v>
+        <v>1.3847749419390085</v>
       </c>
       <c r="G5">
         <f t="shared" si="4"/>
-        <v>0.36901106785318538</v>
+        <v>0.35934980057346</v>
       </c>
       <c r="H5">
         <v>1300</v>
@@ -2264,29 +2264,29 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>0.64139044500673392</v>
+        <v>0.66718928323923199</v>
       </c>
       <c r="B6">
-        <v>92.059659089999997</v>
+        <v>91.209432000000007</v>
       </c>
       <c r="C6">
-        <v>64.033389439999993</v>
+        <v>76.426997</v>
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>1.5616852531865602</v>
+        <v>1.3084381687795479</v>
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>0.56168525318656015</v>
+        <v>0.30843816877954788</v>
       </c>
       <c r="F6">
         <f t="shared" si="3"/>
-        <v>1.5662863561934579</v>
+        <v>0.92676753856234839</v>
       </c>
       <c r="G6">
         <f t="shared" si="4"/>
-        <v>0.35860955499326608</v>
+        <v>0.33281071676076801</v>
       </c>
       <c r="H6">
         <v>1400</v>
@@ -2295,29 +2295,29 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>0.67741140919650833</v>
+        <v>0.69009849387353894</v>
       </c>
       <c r="B7">
-        <v>97.229797980000001</v>
+        <v>94.341280999999995</v>
       </c>
       <c r="C7">
-        <v>73.032066209999996</v>
+        <v>73.074408000000005</v>
       </c>
       <c r="D7">
         <f t="shared" si="1"/>
-        <v>1.3692615475571386</v>
+        <v>1.3684681509838572</v>
       </c>
       <c r="E7">
         <f t="shared" si="2"/>
-        <v>0.36926154755713858</v>
+        <v>0.36846815098385721</v>
       </c>
       <c r="F7">
         <f t="shared" si="3"/>
-        <v>1.1446826021881171</v>
+        <v>1.1889847054615377</v>
       </c>
       <c r="G7">
         <f t="shared" si="4"/>
-        <v>0.32258859080349167</v>
+        <v>0.30990150612646106</v>
       </c>
       <c r="H7">
         <v>1500</v>
@@ -2326,29 +2326,29 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>0.70373163046451825</v>
+        <v>0.7123082376627734</v>
       </c>
       <c r="B8">
-        <v>101.0075758</v>
+        <v>97.377508000000006</v>
       </c>
       <c r="C8">
-        <v>72.890735829999997</v>
+        <v>75.626605999999995</v>
       </c>
       <c r="D8">
         <f t="shared" si="1"/>
-        <v>1.3719164563412531</v>
+        <v>1.3222859690411073</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>0.37191645634125314</v>
+        <v>0.32228596904110729</v>
       </c>
       <c r="F8">
         <f t="shared" si="3"/>
-        <v>1.2553363591408013</v>
+        <v>1.1202474704970178</v>
       </c>
       <c r="G8">
         <f t="shared" si="4"/>
-        <v>0.29626836953548175</v>
+        <v>0.2876917623372266</v>
       </c>
       <c r="H8">
         <v>1600</v>
@@ -2357,29 +2357,29 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>0.72721339574502109</v>
+        <v>0.7344537930689421</v>
       </c>
       <c r="B9">
-        <v>104.3779461</v>
+        <v>100.40496</v>
       </c>
       <c r="C9">
-        <v>72.747359529999997</v>
+        <v>77.453275000000005</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>1.3746203387459224</v>
+        <v>1.291100989596631</v>
       </c>
       <c r="E9">
         <f t="shared" si="2"/>
-        <v>0.37462033874592238</v>
+        <v>0.291100989596631</v>
       </c>
       <c r="F9">
         <f t="shared" si="3"/>
-        <v>1.3733091467928444</v>
+        <v>1.096234787010939</v>
       </c>
       <c r="G9">
         <f t="shared" si="4"/>
-        <v>0.27278660425497891</v>
+        <v>0.2655462069310579</v>
       </c>
       <c r="H9">
         <v>1700</v>
@@ -2388,29 +2388,29 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>0.72994126184330776</v>
+        <v>0.74670204111011751</v>
       </c>
       <c r="B10">
-        <v>104.7694805</v>
+        <v>102.079381</v>
       </c>
       <c r="C10">
-        <v>72.592115849999999</v>
+        <v>78.720592999999994</v>
       </c>
       <c r="D10">
         <f t="shared" si="1"/>
-        <v>1.3775600673581965</v>
+        <v>1.2703156339282151</v>
       </c>
       <c r="E10">
         <f t="shared" si="2"/>
-        <v>0.37756006735819647</v>
+        <v>0.27031563392821512</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>1.3980664722617875</v>
+        <v>1.0671844144063189</v>
       </c>
       <c r="G10">
         <f t="shared" si="4"/>
-        <v>0.27005873815669224</v>
+        <v>0.25329795888988249</v>
       </c>
       <c r="H10">
         <v>1800</v>
@@ -2419,29 +2419,29 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>0.72076236137323757</v>
+        <v>0.76484099056244248</v>
       </c>
       <c r="B11">
-        <v>103.45202020000001</v>
+        <v>104.559102</v>
       </c>
       <c r="C11">
-        <v>72.030764300000001</v>
+        <v>80.309307000000004</v>
       </c>
       <c r="D11">
         <f t="shared" si="1"/>
-        <v>1.388295695204778</v>
+        <v>1.2451856918650785</v>
       </c>
       <c r="E11">
         <f t="shared" si="2"/>
-        <v>0.38829569520477802</v>
+        <v>0.24518569186507855</v>
       </c>
       <c r="F11">
         <f t="shared" si="3"/>
-        <v>1.3905564347068051</v>
+        <v>1.0426378834113241</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>0.27923763862676243</v>
+        <v>0.23515900943755752</v>
       </c>
       <c r="H11">
         <v>1900</v>
@@ -2450,29 +2450,29 @@
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>0.76234831058932162</v>
+        <v>0.79032315687172672</v>
       </c>
       <c r="B12">
-        <v>109.4209091</v>
+        <v>108.042692</v>
       </c>
       <c r="C12">
-        <v>77.615642829999999</v>
+        <v>81.890827999999999</v>
       </c>
       <c r="D12">
         <f t="shared" si="1"/>
-        <v>1.2884000744415403</v>
+        <v>1.2211379765265045</v>
       </c>
       <c r="E12">
         <f t="shared" si="2"/>
-        <v>0.28840007444154026</v>
+        <v>0.22113797652650447</v>
       </c>
       <c r="F12">
         <f t="shared" si="3"/>
-        <v>1.2135410236582211</v>
+        <v>1.0546609402699736</v>
       </c>
       <c r="G12">
         <f t="shared" si="4"/>
-        <v>0.23765168941067838</v>
+        <v>0.20967684312827328</v>
       </c>
       <c r="H12">
         <v>2000</v>
@@ -2481,29 +2481,29 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>0.79662652778702048</v>
+        <v>0.81145060771586064</v>
       </c>
       <c r="B13">
-        <v>114.3409091</v>
+        <v>110.93096199999999</v>
       </c>
       <c r="C13">
-        <v>77.448743890000003</v>
+        <v>76.480919</v>
       </c>
       <c r="D13">
         <f t="shared" si="1"/>
-        <v>1.2911765249805653</v>
+        <v>1.3075156693658452</v>
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>0.29117652498056534</v>
+        <v>0.30751566936584518</v>
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>1.4317330663245771</v>
+        <v>1.630955505295008</v>
       </c>
       <c r="G13">
         <f t="shared" si="4"/>
-        <v>0.20337347221297952</v>
+        <v>0.18854939228413936</v>
       </c>
       <c r="H13">
         <v>2100</v>
@@ -2512,29 +2512,29 @@
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>0.80332567932095322</v>
+        <v>0.83968260435568121</v>
       </c>
       <c r="B14">
-        <v>115.30244759999999</v>
+        <v>114.79047300000001</v>
       </c>
       <c r="C14">
-        <v>77.264830799999999</v>
+        <v>92.520120000000006</v>
       </c>
       <c r="D14">
         <f t="shared" si="1"/>
-        <v>1.2942499059999235</v>
+        <v>1.0808459824738663</v>
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>0.29424990599992351</v>
+        <v>8.0845982473866318E-2</v>
       </c>
       <c r="F14">
         <f t="shared" si="3"/>
-        <v>1.4961277353544824</v>
+        <v>0.50428702480441823</v>
       </c>
       <c r="G14">
         <f t="shared" si="4"/>
-        <v>0.19667432067904678</v>
+        <v>0.16031739564431879</v>
       </c>
       <c r="H14">
         <v>2200</v>
@@ -2543,29 +2543,29 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>0.8326233008217192</v>
+        <v>0.89092461116469701</v>
       </c>
       <c r="B15">
-        <v>119.5075758</v>
+        <v>121.795613</v>
       </c>
       <c r="C15">
-        <v>83.497113569999996</v>
+        <v>83.858969000000002</v>
       </c>
       <c r="D15">
         <f t="shared" si="1"/>
-        <v>1.1976461906813674</v>
+        <v>1.1924782905451652</v>
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>0.19764619068136735</v>
+        <v>0.19247829054516519</v>
       </c>
       <c r="F15">
         <f t="shared" si="3"/>
-        <v>1.1808465076183938</v>
+        <v>1.7646353829257979</v>
       </c>
       <c r="G15">
         <f t="shared" si="4"/>
-        <v>0.1673766991782808</v>
+        <v>0.10907538883530299</v>
       </c>
       <c r="H15">
         <v>2300</v>
@@ -2577,7 +2577,7 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>143.53138530000001</v>
+        <v>136.70697999999999</v>
       </c>
       <c r="C16">
         <v>100</v>

</xml_diff>

<commit_message>
Fix rank-specific perf sheet lookup and dry-run audit
</commit_message>
<xml_diff>
--- a/job_scheduler/data/all_model_data_by_rank.xlsx
+++ b/job_scheduler/data/all_model_data_by_rank.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/imtiazevan/Desktop/Projects/temp/MPR_System_Beta/job_scheduler/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F342CEA1-3B50-994B-8FFE-351B0B4B1026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8428A3E8-4157-BD49-A27A-8FC235F7A696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3400" yWindow="500" windowWidth="28800" windowHeight="16300" activeTab="3" xr2:uid="{15444B7F-6FA5-5E4D-9AAE-4CEB8B7D2F02}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16300" activeTab="2" xr2:uid="{15444B7F-6FA5-5E4D-9AAE-4CEB8B7D2F02}"/>
   </bookViews>
   <sheets>
     <sheet name="comd" sheetId="16" r:id="rId1"/>
-    <sheet name="xsbench" sheetId="15" r:id="rId2"/>
-    <sheet name="minimd" sheetId="14" r:id="rId3"/>
-    <sheet name="hpccg" sheetId="13" r:id="rId4"/>
-    <sheet name="minife" sheetId="6" r:id="rId5"/>
-    <sheet name="swfft" sheetId="5" r:id="rId6"/>
-    <sheet name="simple_moc" sheetId="4" r:id="rId7"/>
-    <sheet name="rsbench" sheetId="9" r:id="rId8"/>
-    <sheet name="aspa" sheetId="10" r:id="rId9"/>
-    <sheet name="cohmm" sheetId="11" r:id="rId10"/>
+    <sheet name="xsbench_rank2" sheetId="15" r:id="rId2"/>
+    <sheet name="xsbench_rank4" sheetId="17" r:id="rId3"/>
+    <sheet name="minimd" sheetId="14" r:id="rId4"/>
+    <sheet name="hpccg" sheetId="13" r:id="rId5"/>
+    <sheet name="minife" sheetId="6" r:id="rId6"/>
+    <sheet name="swfft" sheetId="5" r:id="rId7"/>
+    <sheet name="simple_moc" sheetId="4" r:id="rId8"/>
+    <sheet name="rsbench" sheetId="9" r:id="rId9"/>
+    <sheet name="aspa" sheetId="10" r:id="rId10"/>
+    <sheet name="cohmm" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="12">
   <si>
     <t>Resource</t>
   </si>
@@ -941,6 +942,128 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E99D0987-65F8-5440-830D-42041B7FD317}">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>90.454824360960799</v>
+      </c>
+      <c r="B1">
+        <v>89.469905666732799</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>100.93253560029299</v>
+      </c>
+      <c r="B2">
+        <v>99.840629398258997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>112.159669205404</v>
+      </c>
+      <c r="B3">
+        <v>99.834366004336999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>137.74599752741599</v>
+      </c>
+      <c r="B4">
+        <v>99.485363868592501</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>160.98391727950201</v>
+      </c>
+      <c r="B5">
+        <v>99.583975907782403</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>170.91212494742501</v>
+      </c>
+      <c r="B6">
+        <v>101.586805359571</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>181.08904761817999</v>
+      </c>
+      <c r="B7">
+        <v>99.795911678862595</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>200.67125739453701</v>
+      </c>
+      <c r="B8">
+        <v>99.784987154580193</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>210.32125384406601</v>
+      </c>
+      <c r="B9">
+        <v>96.543899290452103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>221.299308295537</v>
+      </c>
+      <c r="B10">
+        <v>100.21978322102299</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>244.79577512230901</v>
+      </c>
+      <c r="B11">
+        <v>99.537218943853404</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>261.24592378687697</v>
+      </c>
+      <c r="B12">
+        <v>99.862769767471505</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>280.30557715172102</v>
+      </c>
+      <c r="B13">
+        <v>99.740560755831396</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>289.96686227634302</v>
+      </c>
+      <c r="B14">
+        <v>99.958322939862299</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{486C1098-3140-1445-8A34-58E60970723E}">
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1589,6 +1712,516 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F3F29EA-3579-C146-8651-7F0F56939F5A}">
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="5" max="5" width="14.1640625" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" customWidth="1"/>
+    <col min="7" max="7" width="17.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <f t="shared" ref="A2:A15" si="0">B2/$B$16</f>
+        <v>0.80079795768039608</v>
+      </c>
+      <c r="B2">
+        <v>143.159960625076</v>
+      </c>
+      <c r="C2">
+        <v>64.164122664593918</v>
+      </c>
+      <c r="D2">
+        <f t="shared" ref="D2:D15" si="1">1/C2*100</f>
+        <v>1.558503348089578</v>
+      </c>
+      <c r="E2">
+        <f t="shared" ref="E2:E15" si="2">D2-$D$16</f>
+        <v>0.55850334808957802</v>
+      </c>
+      <c r="F2">
+        <f>IFERROR(E2/G2,0)</f>
+        <v>2.8037029218480782</v>
+      </c>
+      <c r="G2">
+        <f>$A$16-A2</f>
+        <v>0.19920204231960392</v>
+      </c>
+      <c r="H2">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <f t="shared" si="0"/>
+        <v>0.8170478870743112</v>
+      </c>
+      <c r="B3">
+        <v>146.06498708010301</v>
+      </c>
+      <c r="C3">
+        <v>67.589347520270408</v>
+      </c>
+      <c r="D3">
+        <f t="shared" si="1"/>
+        <v>1.4795230856461437</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="2"/>
+        <v>0.47952308564614365</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F16" si="3">IFERROR(E3/G3,0)</f>
+        <v>2.6210305963556464</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G16" si="4">$A$16-A3</f>
+        <v>0.1829521129256888</v>
+      </c>
+      <c r="H3">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <f t="shared" si="0"/>
+        <v>0.81762749563889559</v>
+      </c>
+      <c r="B4">
+        <v>146.16860465116201</v>
+      </c>
+      <c r="C4">
+        <v>70.593355848464313</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="1"/>
+        <v>1.4165639074399579</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="2"/>
+        <v>0.41656390743995786</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="3"/>
+        <v>2.2841376714065715</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="4"/>
+        <v>0.18237250436110441</v>
+      </c>
+      <c r="H4">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <f t="shared" si="0"/>
+        <v>0.82658602799033121</v>
+      </c>
+      <c r="B5">
+        <v>147.77013613159301</v>
+      </c>
+      <c r="C5">
+        <v>73.878941654247669</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="1"/>
+        <v>1.3535656813818271</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="2"/>
+        <v>0.35356568138182709</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="3"/>
+        <v>2.0388534861661194</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="4"/>
+        <v>0.17341397200966879</v>
+      </c>
+      <c r="H5">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <f t="shared" si="0"/>
+        <v>0.84263082846150694</v>
+      </c>
+      <c r="B6">
+        <v>150.63849135360701</v>
+      </c>
+      <c r="C6">
+        <v>76.5313344382824</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="1"/>
+        <v>1.3066543362136664</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="2"/>
+        <v>0.30665433621366645</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="3"/>
+        <v>1.9486303017021203</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="4"/>
+        <v>0.15736917153849306</v>
+      </c>
+      <c r="H6">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <f t="shared" si="0"/>
+        <v>0.85462335413143198</v>
+      </c>
+      <c r="B7">
+        <v>152.78241478177699</v>
+      </c>
+      <c r="C7">
+        <v>80.473151574721584</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="1"/>
+        <v>1.2426504746387022</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="2"/>
+        <v>0.24265047463870215</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="3"/>
+        <v>1.6691159242872982</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="4"/>
+        <v>0.14537664586856802</v>
+      </c>
+      <c r="H7">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <f t="shared" si="0"/>
+        <v>0.86985960006581564</v>
+      </c>
+      <c r="B8">
+        <v>155.506223386832</v>
+      </c>
+      <c r="C8">
+        <v>82.512469393307342</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="1"/>
+        <v>1.2119380347633988</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="2"/>
+        <v>0.21193803476339879</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="3"/>
+        <v>1.6285337594673275</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="4"/>
+        <v>0.13014039993418436</v>
+      </c>
+      <c r="H8">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <f t="shared" si="0"/>
+        <v>0.89157283517510011</v>
+      </c>
+      <c r="B9">
+        <v>159.38793394000601</v>
+      </c>
+      <c r="C9">
+        <v>85.892328866764473</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="1"/>
+        <v>1.1642483248430631</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="2"/>
+        <v>0.16424832484306306</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="3"/>
+        <v>1.5148263362627743</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="4"/>
+        <v>0.10842716482489989</v>
+      </c>
+      <c r="H9">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <f t="shared" si="0"/>
+        <v>0.90264352937499504</v>
+      </c>
+      <c r="B10">
+        <v>161.367060048594</v>
+      </c>
+      <c r="C10">
+        <v>88.234379754172522</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="1"/>
+        <v>1.1333450779458909</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="2"/>
+        <v>0.1333450779458909</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="3"/>
+        <v>1.3696580934975127</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="4"/>
+        <v>9.7356470625004965E-2</v>
+      </c>
+      <c r="H10">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <f t="shared" si="0"/>
+        <v>0.91732811849122275</v>
+      </c>
+      <c r="B11">
+        <v>163.99224806201499</v>
+      </c>
+      <c r="C11">
+        <v>90.726266151542035</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="1"/>
+        <v>1.1022166373844577</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="2"/>
+        <v>0.10221663738445774</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="3"/>
+        <v>1.2364135848729345</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="4"/>
+        <v>8.2671881508777245E-2</v>
+      </c>
+      <c r="H11">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <f t="shared" si="0"/>
+        <v>0.92791469886399114</v>
+      </c>
+      <c r="B12">
+        <v>165.884828349944</v>
+      </c>
+      <c r="C12">
+        <v>93.378117863107008</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="1"/>
+        <v>1.0709147098745417</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="2"/>
+        <v>7.0914709874541737E-2</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="3"/>
+        <v>0.983761026963618</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="4"/>
+        <v>7.2085301136008861E-2</v>
+      </c>
+      <c r="H12">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <f t="shared" si="0"/>
+        <v>0.94058103122507652</v>
+      </c>
+      <c r="B13">
+        <v>168.149209302325</v>
+      </c>
+      <c r="C13">
+        <v>94.679733805670793</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="1"/>
+        <v>1.0561922386183404</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="2"/>
+        <v>5.619223861834044E-2</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="3"/>
+        <v>0.94569528514024281</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="4"/>
+        <v>5.9418968774923475E-2</v>
+      </c>
+      <c r="H13">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <f t="shared" si="0"/>
+        <v>0.94853459143898866</v>
+      </c>
+      <c r="B14">
+        <v>169.571080270067</v>
+      </c>
+      <c r="C14">
+        <v>97.603106841941454</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="1"/>
+        <v>1.0245575498118116</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="2"/>
+        <v>2.4557549811811574E-2</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="3"/>
+        <v>0.4771661296091535</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="4"/>
+        <v>5.1465408561011339E-2</v>
+      </c>
+      <c r="H14">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <f t="shared" si="0"/>
+        <v>0.96639843419903504</v>
+      </c>
+      <c r="B15">
+        <v>172.764628657164</v>
+      </c>
+      <c r="C15">
+        <v>97.208638333883655</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="1"/>
+        <v>1.0287151606478513</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="2"/>
+        <v>2.871516064785129E-2</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="3"/>
+        <v>0.85457805204502268</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="4"/>
+        <v>3.3601565800964961E-2</v>
+      </c>
+      <c r="H15">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <f>B16/$B$16</f>
+        <v>1</v>
+      </c>
+      <c r="B16">
+        <v>178.771635531833</v>
+      </c>
+      <c r="C16">
+        <v>100</v>
+      </c>
+      <c r="D16">
+        <f>1/C16*100</f>
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <f>D16-$D$16</f>
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>2400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6C0D575-4C9B-754A-AE7B-6854334B6499}">
   <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2098,7 +2731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0F59526-B852-F242-A3F7-3FC81F3AD9E0}">
   <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2149,7 +2782,7 @@
         <v>53.109729000000002</v>
       </c>
       <c r="D2">
-        <f t="shared" ref="D2:D31" si="1">1/C2*100</f>
+        <f t="shared" ref="D2:D15" si="1">1/C2*100</f>
         <v>1.8828941868635782</v>
       </c>
       <c r="E2">
@@ -2608,7 +3241,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3E71CBB-20F0-7C46-83B1-7FDBC565404C}">
   <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3238,7 +3871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923B1051-F995-914C-8EAE-FF988C233AE2}">
   <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3568,7 +4201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{585258CC-0796-9B4C-A063-C58FA61FB692}">
   <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3864,7 +4497,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9C62D93-16FF-6A4F-83BF-87D1C92809BA}">
   <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4016,126 +4649,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E99D0987-65F8-5440-830D-42041B7FD317}">
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1">
-        <v>90.454824360960799</v>
-      </c>
-      <c r="B1">
-        <v>89.469905666732799</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>100.93253560029299</v>
-      </c>
-      <c r="B2">
-        <v>99.840629398258997</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>112.159669205404</v>
-      </c>
-      <c r="B3">
-        <v>99.834366004336999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>137.74599752741599</v>
-      </c>
-      <c r="B4">
-        <v>99.485363868592501</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>160.98391727950201</v>
-      </c>
-      <c r="B5">
-        <v>99.583975907782403</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>170.91212494742501</v>
-      </c>
-      <c r="B6">
-        <v>101.586805359571</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>181.08904761817999</v>
-      </c>
-      <c r="B7">
-        <v>99.795911678862595</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>200.67125739453701</v>
-      </c>
-      <c r="B8">
-        <v>99.784987154580193</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>210.32125384406601</v>
-      </c>
-      <c r="B9">
-        <v>96.543899290452103</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>221.299308295537</v>
-      </c>
-      <c r="B10">
-        <v>100.21978322102299</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>244.79577512230901</v>
-      </c>
-      <c r="B11">
-        <v>99.537218943853404</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>261.24592378687697</v>
-      </c>
-      <c r="B12">
-        <v>99.862769767471505</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>280.30557715172102</v>
-      </c>
-      <c r="B13">
-        <v>99.740560755831396</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>289.96686227634302</v>
-      </c>
-      <c r="B14">
-        <v>99.958322939862299</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update all model data workbook
</commit_message>
<xml_diff>
--- a/job_scheduler/data/all_model_data_by_rank.xlsx
+++ b/job_scheduler/data/all_model_data_by_rank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/imtiazevan/Desktop/Projects/temp/MPR_System_Beta/job_scheduler/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8428A3E8-4157-BD49-A27A-8FC235F7A696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B757AAC-EE3A-D64F-AB34-94208705006C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16300" activeTab="2" xr2:uid="{15444B7F-6FA5-5E4D-9AAE-4CEB8B7D2F02}"/>
+    <workbookView xWindow="2140" yWindow="580" windowWidth="28800" windowHeight="16300" xr2:uid="{15444B7F-6FA5-5E4D-9AAE-4CEB8B7D2F02}"/>
   </bookViews>
   <sheets>
     <sheet name="comd" sheetId="16" r:id="rId1"/>
@@ -473,29 +473,29 @@
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f t="shared" ref="A2:A15" si="0">B2/$B$16</f>
-        <v>0.52916470421731487</v>
+        <v>0.4459900297270441</v>
       </c>
       <c r="B2">
-        <v>63.121428569999999</v>
+        <v>51.719613870000003</v>
       </c>
       <c r="C2">
-        <v>44.186563579999998</v>
+        <v>43.398477100000001</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:D15" si="1">1/C2*100</f>
-        <v>2.263131411406309</v>
+        <v>2.304228320490997</v>
       </c>
       <c r="E2">
         <f t="shared" ref="E2:E15" si="2">D2-$D$16</f>
-        <v>1.263131411406309</v>
+        <v>1.304228320490997</v>
       </c>
       <c r="F2">
         <f>IFERROR(E2/G2,0)</f>
-        <v>2.6827457982022436</v>
+        <v>2.3541603770206789</v>
       </c>
       <c r="G2">
         <f>$A$16-A2</f>
-        <v>0.47083529578268513</v>
+        <v>0.55400997027295595</v>
       </c>
       <c r="H2">
         <v>1000</v>
@@ -504,29 +504,29 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>0.54781122177644415</v>
+        <v>0.46625058449749396</v>
       </c>
       <c r="B3">
-        <v>65.345679009999998</v>
+        <v>54.069146369999999</v>
       </c>
       <c r="C3">
-        <v>48.697436760000002</v>
+        <v>47.58459173</v>
       </c>
       <c r="D3">
         <f t="shared" si="1"/>
-        <v>2.0534961725570704</v>
+        <v>2.1015206049767237</v>
       </c>
       <c r="E3">
         <f t="shared" si="2"/>
-        <v>1.0534961725570704</v>
+        <v>1.1015206049767237</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F16" si="3">IFERROR(E3/G3,0)</f>
-        <v>2.3297707136735633</v>
+        <v>2.0637410983198574</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G16" si="4">$A$16-A3</f>
-        <v>0.45218877822355585</v>
+        <v>0.53374941550250599</v>
       </c>
       <c r="H3">
         <v>1100</v>
@@ -535,29 +535,29 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>0.58048635512037483</v>
+        <v>0.48555133663735539</v>
       </c>
       <c r="B4">
-        <v>69.243333329999999</v>
+        <v>56.307374539999998</v>
       </c>
       <c r="C4">
-        <v>52.810022529999998</v>
+        <v>51.75781113</v>
       </c>
       <c r="D4">
         <f t="shared" si="1"/>
-        <v>1.893579953373294</v>
+        <v>1.9320755228390587</v>
       </c>
       <c r="E4">
         <f t="shared" si="2"/>
-        <v>0.89357995337329399</v>
+        <v>0.9320755228390587</v>
       </c>
       <c r="F4">
         <f t="shared" si="3"/>
-        <v>2.1300378766695345</v>
+        <v>1.8117950132217975</v>
       </c>
       <c r="G4">
         <f t="shared" si="4"/>
-        <v>0.41951364487962517</v>
+        <v>0.51444866336264461</v>
       </c>
       <c r="H4">
         <v>1200</v>
@@ -566,29 +566,29 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>0.60458743198323062</v>
+        <v>0.50755403485923767</v>
       </c>
       <c r="B5">
-        <v>72.118231050000006</v>
+        <v>58.858936190000001</v>
       </c>
       <c r="C5">
-        <v>56.877634360000002</v>
+        <v>55.535973830000003</v>
       </c>
       <c r="D5">
         <f t="shared" si="1"/>
-        <v>1.7581603230377389</v>
+        <v>1.8006346716113755</v>
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>0.75816032303773895</v>
+        <v>0.80063467161137547</v>
       </c>
       <c r="F5">
         <f t="shared" si="3"/>
-        <v>1.9173905544792533</v>
+        <v>1.6258325345046121</v>
       </c>
       <c r="G5">
         <f t="shared" si="4"/>
-        <v>0.39541256801676938</v>
+        <v>0.49244596514076233</v>
       </c>
       <c r="H5">
         <v>1300</v>
@@ -597,29 +597,29 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>0.64312097437861437</v>
+        <v>0.53137110736465576</v>
       </c>
       <c r="B6">
-        <v>76.714705879999997</v>
+        <v>61.620903300000002</v>
       </c>
       <c r="C6">
-        <v>60.698257640000001</v>
+        <v>59.937136019999997</v>
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>1.6474937483889198</v>
+        <v>1.6684147198263146</v>
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>0.64749374838891982</v>
+        <v>0.66841471982631462</v>
       </c>
       <c r="F6">
         <f t="shared" si="3"/>
-        <v>1.8143227870047161</v>
+        <v>1.4263199096997001</v>
       </c>
       <c r="G6">
         <f t="shared" si="4"/>
-        <v>0.35687902562138563</v>
+        <v>0.46862889263534424</v>
       </c>
       <c r="H6">
         <v>1400</v>
@@ -628,29 +628,29 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>0.66600038874282297</v>
+        <v>0.55646697174877491</v>
       </c>
       <c r="B7">
-        <v>79.443877549999996</v>
+        <v>64.531166600000006</v>
       </c>
       <c r="C7">
-        <v>64.547150180000003</v>
+        <v>64.087651530000002</v>
       </c>
       <c r="D7">
         <f t="shared" si="1"/>
-        <v>1.5492550751060903</v>
+        <v>1.5603629968120942</v>
       </c>
       <c r="E7">
         <f t="shared" si="2"/>
-        <v>0.54925507510609028</v>
+        <v>0.56036299681209423</v>
       </c>
       <c r="F7">
         <f t="shared" si="3"/>
-        <v>1.6444781867819849</v>
+        <v>1.2634075956451536</v>
       </c>
       <c r="G7">
         <f t="shared" si="4"/>
-        <v>0.33399961125717703</v>
+        <v>0.44353302825122509</v>
       </c>
       <c r="H7">
         <v>1500</v>
@@ -659,29 +659,29 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>0.70532974775130175</v>
+        <v>0.58210983060408183</v>
       </c>
       <c r="B8">
-        <v>84.135281390000003</v>
+        <v>67.504862579999994</v>
       </c>
       <c r="C8">
-        <v>68.344158480000004</v>
+        <v>67.709470300000007</v>
       </c>
       <c r="D8">
         <f t="shared" si="1"/>
-        <v>1.4631828414313368</v>
+        <v>1.4768982766654428</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>0.46318284143133681</v>
+        <v>0.47689827666544282</v>
       </c>
       <c r="F8">
         <f t="shared" si="3"/>
-        <v>1.5718683440105652</v>
+        <v>1.1412048226806195</v>
       </c>
       <c r="G8">
         <f t="shared" si="4"/>
-        <v>0.29467025224869825</v>
+        <v>0.41789016939591817</v>
       </c>
       <c r="H8">
         <v>1600</v>
@@ -690,29 +690,29 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>0.7431235686689065</v>
+        <v>0.62295094158761333</v>
       </c>
       <c r="B9">
-        <v>88.643518520000001</v>
+        <v>72.241036820000005</v>
       </c>
       <c r="C9">
-        <v>72.627808819999998</v>
+        <v>72.453343829999994</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>1.376883064830428</v>
+        <v>1.3801985486637272</v>
       </c>
       <c r="E9">
         <f t="shared" si="2"/>
-        <v>0.37688306483042799</v>
+        <v>0.38019854866372715</v>
       </c>
       <c r="F9">
         <f t="shared" si="3"/>
-        <v>1.4671765053628272</v>
+        <v>1.0083529985848574</v>
       </c>
       <c r="G9">
         <f t="shared" si="4"/>
-        <v>0.2568764313310935</v>
+        <v>0.37704905841238667</v>
       </c>
       <c r="H9">
         <v>1700</v>
@@ -721,29 +721,29 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>0.77970743132249387</v>
+        <v>0.64790629909241504</v>
       </c>
       <c r="B10">
-        <v>93.007425740000002</v>
+        <v>75.13500612</v>
       </c>
       <c r="C10">
-        <v>75.76637375</v>
+        <v>75.695414130000003</v>
       </c>
       <c r="D10">
         <f t="shared" si="1"/>
-        <v>1.3198467215807592</v>
+        <v>1.3210839936519678</v>
       </c>
       <c r="E10">
         <f t="shared" si="2"/>
-        <v>0.31984672158075922</v>
+        <v>0.32108399365196783</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>1.4519178903805594</v>
+        <v>0.91192768522786971</v>
       </c>
       <c r="G10">
         <f t="shared" si="4"/>
-        <v>0.22029256867750613</v>
+        <v>0.35209370090758496</v>
       </c>
       <c r="H10">
         <v>1800</v>
@@ -752,29 +752,29 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>0.80252363725320308</v>
+        <v>0.67659497327438256</v>
       </c>
       <c r="B11">
-        <v>95.729057589999996</v>
+        <v>78.461912670000004</v>
       </c>
       <c r="C11">
-        <v>80.55037102</v>
+        <v>80.058675960000002</v>
       </c>
       <c r="D11">
         <f t="shared" si="1"/>
-        <v>1.2414592103513815</v>
+        <v>1.2490838600673755</v>
       </c>
       <c r="E11">
         <f t="shared" si="2"/>
-        <v>0.24145921035138151</v>
+        <v>0.24908386006737548</v>
       </c>
       <c r="F11">
         <f t="shared" si="3"/>
-        <v>1.2227246187483165</v>
+        <v>0.77019167756691254</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>0.19747636274679692</v>
+        <v>0.32340502672561744</v>
       </c>
       <c r="H11">
         <v>1900</v>
@@ -783,29 +783,29 @@
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>0.8381703998506207</v>
+        <v>0.70230659780379723</v>
       </c>
       <c r="B12">
-        <v>99.981182799999999</v>
+        <v>81.44358312</v>
       </c>
       <c r="C12">
-        <v>84.757755810000006</v>
+        <v>84.117726160000004</v>
       </c>
       <c r="D12">
         <f t="shared" si="1"/>
-        <v>1.1798330317306684</v>
+        <v>1.1888100708974276</v>
       </c>
       <c r="E12">
         <f t="shared" si="2"/>
-        <v>0.17983303173066845</v>
+        <v>0.18881007089742763</v>
       </c>
       <c r="F12">
         <f t="shared" si="3"/>
-        <v>1.1112493114032957</v>
+        <v>0.63424338431587857</v>
       </c>
       <c r="G12">
         <f t="shared" si="4"/>
-        <v>0.1618296001493793</v>
+        <v>0.29769340219620277</v>
       </c>
       <c r="H12">
         <v>2000</v>
@@ -814,29 +814,29 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>0.87600634231461061</v>
+        <v>0.72931007702282902</v>
       </c>
       <c r="B13">
-        <v>104.49444440000001</v>
+        <v>84.575064600000005</v>
       </c>
       <c r="C13">
-        <v>88.43826009</v>
+        <v>87.649355799999995</v>
       </c>
       <c r="D13">
         <f t="shared" si="1"/>
-        <v>1.1307323312131434</v>
+        <v>1.1409096973648265</v>
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>0.13073233121314343</v>
+        <v>0.1409096973648265</v>
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>1.0543469210727872</v>
+        <v>0.52055760264378337</v>
       </c>
       <c r="G13">
         <f t="shared" si="4"/>
-        <v>0.12399365768538939</v>
+        <v>0.27068992297717098</v>
       </c>
       <c r="H13">
         <v>2100</v>
@@ -845,29 +845,29 @@
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>0.89525255841864981</v>
+        <v>0.77488963695124724</v>
       </c>
       <c r="B14">
-        <v>106.7902299</v>
+        <v>89.860737110000002</v>
       </c>
       <c r="C14">
-        <v>91.404781060000005</v>
+        <v>91.508404240000004</v>
       </c>
       <c r="D14">
         <f t="shared" si="1"/>
-        <v>1.0940346756517902</v>
+        <v>1.0927958019869848</v>
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>9.4034675651790245E-2</v>
+        <v>9.2795801986984783E-2</v>
       </c>
       <c r="F14">
         <f t="shared" si="3"/>
-        <v>0.89772766028619355</v>
+        <v>0.41222358993258673</v>
       </c>
       <c r="G14">
         <f t="shared" si="4"/>
-        <v>0.10474744158135019</v>
+        <v>0.22511036304875276</v>
       </c>
       <c r="H14">
         <v>2200</v>
@@ -876,29 +876,29 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>0.94413493378470981</v>
+        <v>0.80456485215222684</v>
       </c>
       <c r="B15">
-        <v>112.6211656</v>
+        <v>93.302048729999996</v>
       </c>
       <c r="C15">
-        <v>95.660467749999995</v>
+        <v>94.431522079999993</v>
       </c>
       <c r="D15">
         <f t="shared" si="1"/>
-        <v>1.0453639037323232</v>
+        <v>1.0589684228035903</v>
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>4.5363903732323241E-2</v>
+        <v>5.896842280359027E-2</v>
       </c>
       <c r="F15">
         <f t="shared" si="3"/>
-        <v>0.8120263127855597</v>
+        <v>0.30172885201551103</v>
       </c>
       <c r="G15">
         <f t="shared" si="4"/>
-        <v>5.5865066215290193E-2</v>
+        <v>0.19543514784777316</v>
       </c>
       <c r="H15">
         <v>2300</v>
@@ -910,7 +910,7 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>119.2850318</v>
+        <v>115.9658522</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -1243,29 +1243,29 @@
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f t="shared" ref="A2:A15" si="0">B2/$B$16</f>
-        <v>0.7139325791420843</v>
+        <v>0.63368064814567127</v>
       </c>
       <c r="B2">
-        <v>85.467688940000002</v>
+        <v>74.736948269999999</v>
       </c>
       <c r="C2">
-        <v>62.648231520000003</v>
+        <v>58.742993089999999</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:D15" si="1">1/C2*100</f>
-        <v>1.5962142517634468</v>
+        <v>1.7023306906883386</v>
       </c>
       <c r="E2">
         <f t="shared" ref="E2:E15" si="2">D2-$D$16</f>
-        <v>0.59621425176344678</v>
+        <v>0.70233069068833864</v>
       </c>
       <c r="F2">
         <f>IFERROR(E2/G2,0)</f>
-        <v>2.0841738985005747</v>
+        <v>1.9172634127383716</v>
       </c>
       <c r="G2">
         <f>$A$16-A2</f>
-        <v>0.2860674208579157</v>
+        <v>0.36631935185432873</v>
       </c>
       <c r="H2">
         <v>1000</v>
@@ -1274,29 +1274,29 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>0.73099715886243366</v>
+        <v>0.65326406531574643</v>
       </c>
       <c r="B3">
-        <v>87.510557180000006</v>
+        <v>77.046636660000004</v>
       </c>
       <c r="C3">
-        <v>66.037876049999994</v>
+        <v>62.292301530000003</v>
       </c>
       <c r="D3">
         <f t="shared" si="1"/>
-        <v>1.5142824993990702</v>
+        <v>1.6053348093398017</v>
       </c>
       <c r="E3">
         <f t="shared" si="2"/>
-        <v>0.51428249939907023</v>
+        <v>0.60533480933980166</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F16" si="3">IFERROR(E3/G3,0)</f>
-        <v>1.9118106605278173</v>
+        <v>1.7458092709399582</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G16" si="4">$A$16-A3</f>
-        <v>0.26900284113756634</v>
+        <v>0.34673593468425357</v>
       </c>
       <c r="H3">
         <v>1100</v>
@@ -1305,29 +1305,29 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>0.7386914039486483</v>
+        <v>0.67374736796325019</v>
       </c>
       <c r="B4">
-        <v>88.431665649999999</v>
+        <v>79.462458470000001</v>
       </c>
       <c r="C4">
-        <v>69.008215539999995</v>
+        <v>66.316953170000005</v>
       </c>
       <c r="D4">
         <f t="shared" si="1"/>
-        <v>1.4491028237360506</v>
+        <v>1.5079100474301841</v>
       </c>
       <c r="E4">
         <f t="shared" si="2"/>
-        <v>0.44910282373605059</v>
+        <v>0.50791004743018409</v>
       </c>
       <c r="F4">
         <f t="shared" si="3"/>
-        <v>1.7186683887268448</v>
+        <v>1.556799846362533</v>
       </c>
       <c r="G4">
         <f t="shared" si="4"/>
-        <v>0.2613085960513517</v>
+        <v>0.32625263203674981</v>
       </c>
       <c r="H4">
         <v>1200</v>
@@ -1336,29 +1336,29 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>0.76510807865768038</v>
+        <v>0.6904271179337903</v>
       </c>
       <c r="B5">
-        <v>91.594110119999996</v>
+        <v>81.429685359999993</v>
       </c>
       <c r="C5">
-        <v>72.272877159999993</v>
+        <v>68.437443500000001</v>
       </c>
       <c r="D5">
         <f t="shared" si="1"/>
-        <v>1.3836449291843858</v>
+        <v>1.4611884209263311</v>
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>0.38364492918438575</v>
+        <v>0.46118842092633106</v>
       </c>
       <c r="F5">
         <f t="shared" si="3"/>
-        <v>1.6332827752951156</v>
+        <v>1.4897571707449966</v>
       </c>
       <c r="G5">
         <f t="shared" si="4"/>
-        <v>0.23489192134231962</v>
+        <v>0.3095728820662097</v>
       </c>
       <c r="H5">
         <v>1300</v>
@@ -1367,29 +1367,29 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>0.78353895178220911</v>
+        <v>0.71495410266889659</v>
       </c>
       <c r="B6">
-        <v>93.800542739999997</v>
+        <v>84.322423200000003</v>
       </c>
       <c r="C6">
-        <v>75.879306600000007</v>
+        <v>71.588234189999994</v>
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>1.3178823645180753</v>
+        <v>1.3968775893339298</v>
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>0.31788236451807528</v>
+        <v>0.3968775893339298</v>
       </c>
       <c r="F6">
         <f t="shared" si="3"/>
-        <v>1.4685430341178058</v>
+        <v>1.3923287198655065</v>
       </c>
       <c r="G6">
         <f t="shared" si="4"/>
-        <v>0.21646104821779089</v>
+        <v>0.28504589733110341</v>
       </c>
       <c r="H6">
         <v>1400</v>
@@ -1398,29 +1398,29 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>0.80058999097530403</v>
+        <v>0.73330554577427853</v>
       </c>
       <c r="B7">
-        <v>95.841789989999995</v>
+        <v>86.486811299999999</v>
       </c>
       <c r="C7">
-        <v>78.794143480000002</v>
+        <v>76.051251699999995</v>
       </c>
       <c r="D7">
         <f t="shared" si="1"/>
-        <v>1.2691298564008453</v>
+        <v>1.3149027499832722</v>
       </c>
       <c r="E7">
         <f t="shared" si="2"/>
-        <v>0.2691298564008453</v>
+        <v>0.31490274998327217</v>
       </c>
       <c r="F7">
         <f t="shared" si="3"/>
-        <v>1.3496306314670237</v>
+        <v>1.1807622730570497</v>
       </c>
       <c r="G7">
         <f t="shared" si="4"/>
-        <v>0.19941000902469597</v>
+        <v>0.26669445422572147</v>
       </c>
       <c r="H7">
         <v>1500</v>
@@ -1429,29 +1429,29 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>0.81969336250235403</v>
+        <v>0.75808373638765381</v>
       </c>
       <c r="B8">
-        <v>98.128730050000001</v>
+        <v>89.409176619999997</v>
       </c>
       <c r="C8">
-        <v>79.717777139999995</v>
+        <v>77.855184820000005</v>
       </c>
       <c r="D8">
         <f t="shared" si="1"/>
-        <v>1.2544253438524817</v>
+        <v>1.2844359721346557</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>0.25442534385248172</v>
+        <v>0.28443597213465566</v>
       </c>
       <c r="F8">
         <f t="shared" si="3"/>
-        <v>1.4110703154552666</v>
+        <v>1.1757620917560314</v>
       </c>
       <c r="G8">
         <f t="shared" si="4"/>
-        <v>0.18030663749764597</v>
+        <v>0.24191626361234619</v>
       </c>
       <c r="H8">
         <v>1600</v>
@@ -1460,29 +1460,29 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>0.86117817908636085</v>
+        <v>0.80331967509807201</v>
       </c>
       <c r="B9">
-        <v>103.09504130000001</v>
+        <v>94.744349819999996</v>
       </c>
       <c r="C9">
-        <v>84.121420619999995</v>
+        <v>80.883177149999995</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>1.1887578605184046</v>
+        <v>1.2363510376768132</v>
       </c>
       <c r="E9">
         <f t="shared" si="2"/>
-        <v>0.1887578605184046</v>
+        <v>0.2363510376768132</v>
       </c>
       <c r="F9">
         <f t="shared" si="3"/>
-        <v>1.3597131868471211</v>
+        <v>1.2017014807895323</v>
       </c>
       <c r="G9">
         <f t="shared" si="4"/>
-        <v>0.13882182091363915</v>
+        <v>0.19668032490192799</v>
       </c>
       <c r="H9">
         <v>1700</v>
@@ -1491,29 +1491,29 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>0.86307274693228786</v>
+        <v>0.82335366286300338</v>
       </c>
       <c r="B10">
-        <v>103.3218475</v>
+        <v>97.107178970000007</v>
       </c>
       <c r="C10">
-        <v>85.101221260000003</v>
+        <v>84.183755329999997</v>
       </c>
       <c r="D10">
         <f t="shared" si="1"/>
-        <v>1.1750712683015614</v>
+        <v>1.1878776327808185</v>
       </c>
       <c r="E10">
         <f t="shared" si="2"/>
-        <v>0.17507126830156139</v>
+        <v>0.18787763278081848</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>1.2785713901306892</v>
+        <v>1.0635806879771954</v>
       </c>
       <c r="G10">
         <f t="shared" si="4"/>
-        <v>0.13692725306771214</v>
+        <v>0.17664633713699662</v>
       </c>
       <c r="H10">
         <v>1800</v>
@@ -1522,29 +1522,29 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>0.89761447583613185</v>
+        <v>0.84184321083328106</v>
       </c>
       <c r="B11">
-        <v>107.4569743</v>
+        <v>99.287855300000004</v>
       </c>
       <c r="C11">
-        <v>87.608318639999993</v>
+        <v>86.469658429999996</v>
       </c>
       <c r="D11">
         <f t="shared" si="1"/>
-        <v>1.1414441180057329</v>
+        <v>1.1564750204368306</v>
       </c>
       <c r="E11">
         <f t="shared" si="2"/>
-        <v>0.14144411800573287</v>
+        <v>0.15647502043683059</v>
       </c>
       <c r="F11">
         <f t="shared" si="3"/>
-        <v>1.3814855094100158</v>
+        <v>0.98936644617819391</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>0.10238552416386815</v>
+        <v>0.15815678916671894</v>
       </c>
       <c r="H11">
         <v>1900</v>
@@ -1553,29 +1553,29 @@
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>0.91283614802257584</v>
+        <v>0.86700797921385619</v>
       </c>
       <c r="B12">
-        <v>109.2792208</v>
+        <v>102.255814</v>
       </c>
       <c r="C12">
-        <v>91.430319229999995</v>
+        <v>90.299367430000004</v>
       </c>
       <c r="D12">
         <f t="shared" si="1"/>
-        <v>1.0937290916423721</v>
+        <v>1.1074274698271827</v>
       </c>
       <c r="E12">
         <f t="shared" si="2"/>
-        <v>9.3729091642372087E-2</v>
+        <v>0.10742746982718265</v>
       </c>
       <c r="F12">
         <f t="shared" si="3"/>
-        <v>1.0753206692454156</v>
+        <v>0.80777379869977373</v>
       </c>
       <c r="G12">
         <f t="shared" si="4"/>
-        <v>8.7163851977424156E-2</v>
+        <v>0.13299202078614381</v>
       </c>
       <c r="H12">
         <v>2000</v>
@@ -1584,29 +1584,29 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>0.93835940496217762</v>
+        <v>0.88573868897510788</v>
       </c>
       <c r="B13">
-        <v>112.3347107</v>
+        <v>104.4649332</v>
       </c>
       <c r="C13">
-        <v>94.291037660000001</v>
+        <v>92.529920869999998</v>
       </c>
       <c r="D13">
         <f t="shared" si="1"/>
-        <v>1.0605461821364794</v>
+        <v>1.0807314980901701</v>
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>6.0546182136479443E-2</v>
+        <v>8.0731498090170106E-2</v>
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>0.98224525735562085</v>
+        <v>0.70655147718883204</v>
       </c>
       <c r="G13">
         <f t="shared" si="4"/>
-        <v>6.1640595037822377E-2</v>
+        <v>0.11426131102489212</v>
       </c>
       <c r="H13">
         <v>2100</v>
@@ -1615,29 +1615,29 @@
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>0.95563658613826807</v>
+        <v>0.91294323605020511</v>
       </c>
       <c r="B14">
-        <v>114.4030303</v>
+        <v>107.67346550000001</v>
       </c>
       <c r="C14">
-        <v>94.292639129999998</v>
+        <v>94.221278690000005</v>
       </c>
       <c r="D14">
         <f t="shared" si="1"/>
-        <v>1.0605281697771907</v>
+        <v>1.0613313827868196</v>
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>6.0528169777190666E-2</v>
+        <v>6.1331382786819599E-2</v>
       </c>
       <c r="F14">
         <f t="shared" si="3"/>
-        <v>1.3643713255665955</v>
+        <v>0.70449876614054985</v>
       </c>
       <c r="G14">
         <f t="shared" si="4"/>
-        <v>4.4363413861731926E-2</v>
+        <v>8.7056763949794891E-2</v>
       </c>
       <c r="H14">
         <v>2200</v>
@@ -1646,29 +1646,29 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>0.97570797217151051</v>
+        <v>0.93022578311400694</v>
       </c>
       <c r="B15">
-        <v>116.8058552</v>
+        <v>109.71178690000001</v>
       </c>
       <c r="C15">
-        <v>97.063090180000003</v>
+        <v>96.892781290000002</v>
       </c>
       <c r="D15">
         <f t="shared" si="1"/>
-        <v>1.0302577407596814</v>
+        <v>1.032068629557656</v>
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>3.0257740759681351E-2</v>
+        <v>3.2068629557655992E-2</v>
       </c>
       <c r="F15">
         <f t="shared" si="3"/>
-        <v>1.245583158940536</v>
+        <v>0.45960572527892696</v>
       </c>
       <c r="G15">
         <f t="shared" si="4"/>
-        <v>2.4292027828489493E-2</v>
+        <v>6.9774216885993057E-2</v>
       </c>
       <c r="H15">
         <v>2300</v>
@@ -1680,7 +1680,7 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>119.71394979999999</v>
+        <v>117.9410299</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -2263,29 +2263,29 @@
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f t="shared" ref="A2:A15" si="0">B2/$B$16</f>
-        <v>0.58844289833337582</v>
+        <v>0.46771966375263374</v>
       </c>
       <c r="B2">
-        <v>68.435314689999998</v>
+        <v>53.146489889999998</v>
       </c>
       <c r="C2">
-        <v>42.937385480000003</v>
+        <v>42.754730700000003</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:D15" si="1">1/C2*100</f>
-        <v>2.3289727327850329</v>
+        <v>2.3389224622107139</v>
       </c>
       <c r="E2">
         <f t="shared" ref="E2:E15" si="2">D2-$D$16</f>
-        <v>1.3289727327850329</v>
+        <v>1.3389224622107139</v>
       </c>
       <c r="F2">
         <f>IFERROR(E2/G2,0)</f>
-        <v>3.2291332779905422</v>
+        <v>2.515446036669815</v>
       </c>
       <c r="G2">
         <f>$A$16-A2</f>
-        <v>0.41155710166662418</v>
+        <v>0.53228033624736626</v>
       </c>
       <c r="H2">
         <v>1000</v>
@@ -2294,29 +2294,29 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>0.61019604564940422</v>
+        <v>0.4884151984252505</v>
       </c>
       <c r="B3">
-        <v>70.965183749999994</v>
+        <v>55.498101570000003</v>
       </c>
       <c r="C3">
-        <v>46.379192860000003</v>
+        <v>46.955052090000002</v>
       </c>
       <c r="D3">
         <f t="shared" si="1"/>
-        <v>2.1561392907776447</v>
+        <v>2.1296962850414336</v>
       </c>
       <c r="E3">
         <f t="shared" si="2"/>
-        <v>1.1561392907776447</v>
+        <v>1.1296962850414336</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F16" si="3">IFERROR(E3/G3,0)</f>
-        <v>2.9659506474318493</v>
+        <v>2.2082287854604483</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G16" si="4">$A$16-A3</f>
-        <v>0.38980395435059578</v>
+        <v>0.5115848015747495</v>
       </c>
       <c r="H3">
         <v>1100</v>
@@ -2325,29 +2325,29 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>0.62090050027167099</v>
+        <v>0.50756114063427249</v>
       </c>
       <c r="B4">
-        <v>72.210101010000002</v>
+        <v>57.673634700000001</v>
       </c>
       <c r="C4">
-        <v>49.301012890000003</v>
+        <v>50.95280477</v>
       </c>
       <c r="D4">
         <f t="shared" si="1"/>
-        <v>2.028355892466533</v>
+        <v>1.9626004976840454</v>
       </c>
       <c r="E4">
         <f t="shared" si="2"/>
-        <v>1.028355892466533</v>
+        <v>0.96260049768404543</v>
       </c>
       <c r="F4">
         <f t="shared" si="3"/>
-        <v>2.7126279333090002</v>
+        <v>1.9547614477945483</v>
       </c>
       <c r="G4">
         <f t="shared" si="4"/>
-        <v>0.37909949972832901</v>
+        <v>0.49243885936572751</v>
       </c>
       <c r="H4">
         <v>1200</v>
@@ -2356,29 +2356,29 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>0.64656869560652996</v>
+        <v>0.52496452466265442</v>
       </c>
       <c r="B5">
-        <v>75.195286199999998</v>
+        <v>59.651162790000001</v>
       </c>
       <c r="C5">
-        <v>55.207013519999997</v>
+        <v>54.40340088</v>
       </c>
       <c r="D5">
         <f t="shared" si="1"/>
-        <v>1.8113640572818293</v>
+        <v>1.8381203818594805</v>
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>0.81136405728182925</v>
+        <v>0.83812038185948046</v>
       </c>
       <c r="F5">
         <f t="shared" si="3"/>
-        <v>2.2956768322325778</v>
+        <v>1.7643321927994762</v>
       </c>
       <c r="G5">
         <f t="shared" si="4"/>
-        <v>0.35343130439347004</v>
+        <v>0.47503547533734558</v>
       </c>
       <c r="H5">
         <v>1300</v>
@@ -2387,29 +2387,29 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>0.65870257562744328</v>
+        <v>0.5467945220814634</v>
       </c>
       <c r="B6">
-        <v>76.606444190000005</v>
+        <v>62.131682269999999</v>
       </c>
       <c r="C6">
-        <v>57.913245250000003</v>
+        <v>58.393668750000003</v>
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>1.7267207107513975</v>
+        <v>1.7125144239203158</v>
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>0.72672071075139755</v>
+        <v>0.71251442392031583</v>
       </c>
       <c r="F6">
         <f t="shared" si="3"/>
-        <v>2.1292885877688805</v>
+        <v>1.5721663983249334</v>
       </c>
       <c r="G6">
         <f t="shared" si="4"/>
-        <v>0.34129742437255672</v>
+        <v>0.4532054779185366</v>
       </c>
       <c r="H6">
         <v>1400</v>
@@ -2418,29 +2418,29 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>0.67482910021387899</v>
+        <v>0.57677635982465547</v>
       </c>
       <c r="B7">
-        <v>78.481942709999998</v>
+        <v>65.538486730000002</v>
       </c>
       <c r="C7">
-        <v>62.587173579999998</v>
+        <v>63.0438081</v>
       </c>
       <c r="D7">
         <f t="shared" si="1"/>
-        <v>1.5977714646624568</v>
+        <v>1.5861985976700541</v>
       </c>
       <c r="E7">
         <f t="shared" si="2"/>
-        <v>0.59777146466245679</v>
+        <v>0.58619859767005411</v>
       </c>
       <c r="F7">
         <f t="shared" si="3"/>
-        <v>1.8383301367239102</v>
+        <v>1.3850799955956805</v>
       </c>
       <c r="G7">
         <f t="shared" si="4"/>
-        <v>0.32517089978612101</v>
+        <v>0.42322364017534453</v>
       </c>
       <c r="H7">
         <v>1500</v>
@@ -2449,29 +2449,29 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>0.71834485253770897</v>
+        <v>0.61454649582467369</v>
       </c>
       <c r="B8">
-        <v>83.542780750000006</v>
+        <v>69.830267269999993</v>
       </c>
       <c r="C8">
-        <v>66.146698259999994</v>
+        <v>66.526441109999993</v>
       </c>
       <c r="D8">
         <f t="shared" si="1"/>
-        <v>1.5117912553538846</v>
+        <v>1.503161725345449</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>0.51179125535388459</v>
+        <v>0.50316172534544901</v>
       </c>
       <c r="F8">
         <f t="shared" si="3"/>
-        <v>1.8170846865932211</v>
+        <v>1.3053759270445815</v>
       </c>
       <c r="G8">
         <f t="shared" si="4"/>
-        <v>0.28165514746229103</v>
+        <v>0.38545350417532631</v>
       </c>
       <c r="H8">
         <v>1600</v>
@@ -2480,29 +2480,29 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>0.73505191681806692</v>
+        <v>0.64593750634686453</v>
       </c>
       <c r="B9">
-        <v>85.485795449999998</v>
+        <v>73.397194540000001</v>
       </c>
       <c r="C9">
-        <v>70.041843220000004</v>
+        <v>70.446483270000002</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>1.427717995454546</v>
+        <v>1.4195172755001884</v>
       </c>
       <c r="E9">
         <f t="shared" si="2"/>
-        <v>0.42771799545454603</v>
+        <v>0.41951727550018836</v>
       </c>
       <c r="F9">
         <f t="shared" si="3"/>
-        <v>1.6143464422078608</v>
+        <v>1.1848678779039978</v>
       </c>
       <c r="G9">
         <f t="shared" si="4"/>
-        <v>0.26494808318193308</v>
+        <v>0.35406249365313547</v>
       </c>
       <c r="H9">
         <v>1700</v>
@@ -2511,29 +2511,29 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>0.75427320732043612</v>
+        <v>0.66430696019355473</v>
       </c>
       <c r="B10">
-        <v>87.721212120000004</v>
+        <v>75.484496120000003</v>
       </c>
       <c r="C10">
-        <v>74.724498550000007</v>
+        <v>74.886436939999996</v>
       </c>
       <c r="D10">
         <f t="shared" si="1"/>
-        <v>1.3382491945809114</v>
+        <v>1.3353552937779818</v>
       </c>
       <c r="E10">
         <f t="shared" si="2"/>
-        <v>0.33824919458091141</v>
+        <v>0.33535529377798179</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>1.376525493587506</v>
+        <v>0.99899388432760416</v>
       </c>
       <c r="G10">
         <f t="shared" si="4"/>
-        <v>0.24572679267956388</v>
+        <v>0.33569303980644527</v>
       </c>
       <c r="H10">
         <v>1800</v>
@@ -2542,29 +2542,29 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>0.77480544747190461</v>
+        <v>0.67853455627482984</v>
       </c>
       <c r="B11">
-        <v>90.109090910000006</v>
+        <v>77.101162790000004</v>
       </c>
       <c r="C11">
-        <v>79.691496670000006</v>
+        <v>74.830950169999994</v>
       </c>
       <c r="D11">
         <f t="shared" si="1"/>
-        <v>1.2548390252236932</v>
+        <v>1.336345452955245</v>
       </c>
       <c r="E11">
         <f t="shared" si="2"/>
-        <v>0.25483902522369317</v>
+        <v>0.33634545295524498</v>
       </c>
       <c r="F11">
         <f t="shared" si="3"/>
-        <v>1.1316393863119727</v>
+        <v>1.0462880521702238</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>0.22519455252809539</v>
+        <v>0.32146544372517016</v>
       </c>
       <c r="H11">
         <v>1900</v>
@@ -2573,29 +2573,29 @@
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>0.79681544310644103</v>
+        <v>0.70867652523022817</v>
       </c>
       <c r="B12">
-        <v>92.668831170000004</v>
+        <v>80.526162790000001</v>
       </c>
       <c r="C12">
-        <v>79.447820460000003</v>
+        <v>82.867839419999996</v>
       </c>
       <c r="D12">
         <f t="shared" si="1"/>
-        <v>1.258687770425968</v>
+        <v>1.2067407657772864</v>
       </c>
       <c r="E12">
         <f t="shared" si="2"/>
-        <v>0.25868777042596802</v>
+        <v>0.20674076577728639</v>
       </c>
       <c r="F12">
         <f t="shared" si="3"/>
-        <v>1.273166496415794</v>
+        <v>0.70966051033364286</v>
       </c>
       <c r="G12">
         <f t="shared" si="4"/>
-        <v>0.20318455689355897</v>
+        <v>0.29132347476977183</v>
       </c>
       <c r="H12">
         <v>2000</v>
@@ -2604,29 +2604,29 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>0.81595330734682503</v>
+        <v>0.74115977923673426</v>
       </c>
       <c r="B13">
-        <v>94.894545449999995</v>
+        <v>84.21720053</v>
       </c>
       <c r="C13">
-        <v>85.297601810000003</v>
+        <v>85.523796709999999</v>
       </c>
       <c r="D13">
         <f t="shared" si="1"/>
-        <v>1.17236590335505</v>
+        <v>1.1692652085955317</v>
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>0.17236590335504998</v>
+        <v>0.16926520859553174</v>
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>0.93653355499228264</v>
+        <v>0.65393704307778755</v>
       </c>
       <c r="G13">
         <f t="shared" si="4"/>
-        <v>0.18404669265317497</v>
+        <v>0.25884022076326574</v>
       </c>
       <c r="H13">
         <v>2100</v>
@@ -2635,29 +2635,29 @@
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>0.84174888822486671</v>
+        <v>0.77983607549360523</v>
       </c>
       <c r="B14">
-        <v>97.894545449999995</v>
+        <v>88.611947099999995</v>
       </c>
       <c r="C14">
-        <v>88.552910580000002</v>
+        <v>88.679847289999998</v>
       </c>
       <c r="D14">
         <f t="shared" si="1"/>
-        <v>1.1292683588266534</v>
+        <v>1.1276519193022621</v>
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>0.12926835882665344</v>
+        <v>0.12765191930226205</v>
       </c>
       <c r="F14">
         <f t="shared" si="3"/>
-        <v>0.81685592838258947</v>
+        <v>0.57980397827871355</v>
       </c>
       <c r="G14">
         <f t="shared" si="4"/>
-        <v>0.15825111177513329</v>
+        <v>0.22016392450639477</v>
       </c>
       <c r="H14">
         <v>2200</v>
@@ -2666,29 +2666,29 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>0.86955577676947649</v>
+        <v>0.79602223088930213</v>
       </c>
       <c r="B15">
-        <v>101.12845849999999</v>
+        <v>90.451162789999998</v>
       </c>
       <c r="C15">
-        <v>96.015000229999998</v>
+        <v>92.046921830000002</v>
       </c>
       <c r="D15">
         <f t="shared" si="1"/>
-        <v>1.0415039291824622</v>
+        <v>1.0864024348873764</v>
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>4.1503929182462151E-2</v>
+        <v>8.6402434887376423E-2</v>
       </c>
       <c r="F15">
         <f t="shared" si="3"/>
-        <v>0.3181737615863266</v>
+        <v>0.42358750791360106</v>
       </c>
       <c r="G15">
         <f t="shared" si="4"/>
-        <v>0.13044422323052351</v>
+        <v>0.20397776911069787</v>
       </c>
       <c r="H15">
         <v>2300</v>
@@ -2700,7 +2700,7 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>116.2989899</v>
+        <v>113.62894060000001</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -2773,29 +2773,29 @@
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f t="shared" ref="A2:A15" si="0">B2/$B$16</f>
-        <v>0.5853651583847439</v>
+        <v>0.55702894007674031</v>
       </c>
       <c r="B2">
-        <v>80.023503000000005</v>
+        <v>43.173611110000003</v>
       </c>
       <c r="C2">
-        <v>53.109729000000002</v>
+        <v>49.735794980000001</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:D15" si="1">1/C2*100</f>
-        <v>1.8828941868635782</v>
+        <v>2.0106243408839144</v>
       </c>
       <c r="E2">
         <f t="shared" ref="E2:E15" si="2">D2-$D$16</f>
-        <v>0.88289418686357823</v>
+        <v>1.0106243408839144</v>
       </c>
       <c r="F2">
         <f>IFERROR(E2/G2,0)</f>
-        <v>2.1293294683682777</v>
+        <v>2.2814680964914387</v>
       </c>
       <c r="G2">
         <f>$A$16-A2</f>
-        <v>0.4146348416152561</v>
+        <v>0.44297105992325969</v>
       </c>
       <c r="H2">
         <v>1000</v>
@@ -2804,29 +2804,29 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>0.60720817620285383</v>
+        <v>0.56614722973589593</v>
       </c>
       <c r="B3">
-        <v>83.009596000000002</v>
+        <v>43.880341880000003</v>
       </c>
       <c r="C3">
-        <v>60.344082</v>
+        <v>54.339077150000001</v>
       </c>
       <c r="D3">
         <f t="shared" si="1"/>
-        <v>1.6571633321060382</v>
+        <v>1.840296251700329</v>
       </c>
       <c r="E3">
         <f t="shared" si="2"/>
-        <v>0.65716333210603817</v>
+        <v>0.84029625170032896</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F16" si="3">IFERROR(E3/G3,0)</f>
-        <v>1.6730575645724854</v>
+        <v>1.9368235246920424</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G16" si="4">$A$16-A3</f>
-        <v>0.39279182379714617</v>
+        <v>0.43385277026410407</v>
       </c>
       <c r="H3">
         <v>1100</v>
@@ -2835,29 +2835,29 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>0.61983106495366957</v>
+        <v>0.58242988981388366</v>
       </c>
       <c r="B4">
-        <v>84.735232999999994</v>
+        <v>45.142361110000003</v>
       </c>
       <c r="C4">
-        <v>62.392927</v>
+        <v>58.672117669999999</v>
       </c>
       <c r="D4">
         <f t="shared" si="1"/>
-        <v>1.6027457727700449</v>
+        <v>1.7043870917093491</v>
       </c>
       <c r="E4">
         <f t="shared" si="2"/>
-        <v>0.60274577277004493</v>
+        <v>0.7043870917093491</v>
       </c>
       <c r="F4">
         <f t="shared" si="3"/>
-        <v>1.5854682411033652</v>
+        <v>1.6868714367400357</v>
       </c>
       <c r="G4">
         <f t="shared" si="4"/>
-        <v>0.38016893504633043</v>
+        <v>0.41757011018611634</v>
       </c>
       <c r="H4">
         <v>1200</v>
@@ -2866,29 +2866,29 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>0.64065019942654</v>
+        <v>0.59145513568125907</v>
       </c>
       <c r="B5">
-        <v>87.581354000000005</v>
+        <v>45.841880340000003</v>
       </c>
       <c r="C5">
-        <v>66.772675000000007</v>
+        <v>62.377502839999998</v>
       </c>
       <c r="D5">
         <f t="shared" si="1"/>
-        <v>1.4976185992249074</v>
+        <v>1.6031420856410801</v>
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>0.49761859922490737</v>
+        <v>0.60314208564108007</v>
       </c>
       <c r="F5">
         <f t="shared" si="3"/>
-        <v>1.3847749419390085</v>
+        <v>1.4763178742849576</v>
       </c>
       <c r="G5">
         <f t="shared" si="4"/>
-        <v>0.35934980057346</v>
+        <v>0.40854486431874093</v>
       </c>
       <c r="H5">
         <v>1300</v>
@@ -2897,29 +2897,29 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>0.66718928323923199</v>
+        <v>0.61063893709083494</v>
       </c>
       <c r="B6">
-        <v>91.209432000000007</v>
+        <v>47.32875817</v>
       </c>
       <c r="C6">
-        <v>76.426997</v>
+        <v>65.073609640000001</v>
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>1.3084381687795479</v>
+        <v>1.5367212692398602</v>
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>0.30843816877954788</v>
+        <v>0.53672126923986019</v>
       </c>
       <c r="F6">
         <f t="shared" si="3"/>
-        <v>0.92676753856234839</v>
+        <v>1.3784667250229721</v>
       </c>
       <c r="G6">
         <f t="shared" si="4"/>
-        <v>0.33281071676076801</v>
+        <v>0.38936106290916506</v>
       </c>
       <c r="H6">
         <v>1400</v>
@@ -2928,29 +2928,29 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>0.69009849387353894</v>
+        <v>0.65596548422003575</v>
       </c>
       <c r="B7">
-        <v>94.341280999999995</v>
+        <v>50.841880340000003</v>
       </c>
       <c r="C7">
-        <v>73.074408000000005</v>
+        <v>69.716540129999998</v>
       </c>
       <c r="D7">
         <f t="shared" si="1"/>
-        <v>1.3684681509838572</v>
+        <v>1.4343798446327172</v>
       </c>
       <c r="E7">
         <f t="shared" si="2"/>
-        <v>0.36846815098385721</v>
+        <v>0.43437984463271717</v>
       </c>
       <c r="F7">
         <f t="shared" si="3"/>
-        <v>1.1889847054615377</v>
+        <v>1.2626054209936759</v>
       </c>
       <c r="G7">
         <f t="shared" si="4"/>
-        <v>0.30990150612646106</v>
+        <v>0.34403451577996425</v>
       </c>
       <c r="H7">
         <v>1500</v>
@@ -2959,29 +2959,29 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>0.7123082376627734</v>
+        <v>0.66939214356674237</v>
       </c>
       <c r="B8">
-        <v>97.377508000000006</v>
+        <v>51.882539680000001</v>
       </c>
       <c r="C8">
-        <v>75.626605999999995</v>
+        <v>75.13189509</v>
       </c>
       <c r="D8">
         <f t="shared" si="1"/>
-        <v>1.3222859690411073</v>
+        <v>1.3309926480652545</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>0.32228596904110729</v>
+        <v>0.33099264806525452</v>
       </c>
       <c r="F8">
         <f t="shared" si="3"/>
-        <v>1.1202474704970178</v>
+        <v>1.0011638913731458</v>
       </c>
       <c r="G8">
         <f t="shared" si="4"/>
-        <v>0.2876917623372266</v>
+        <v>0.33060785643325763</v>
       </c>
       <c r="H8">
         <v>1600</v>
@@ -2990,29 +2990,29 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>0.7344537930689421</v>
+        <v>0.72835255418565947</v>
       </c>
       <c r="B9">
-        <v>100.40496</v>
+        <v>56.452380949999998</v>
       </c>
       <c r="C9">
-        <v>77.453275000000005</v>
+        <v>76.961307410000003</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>1.291100989596631</v>
+        <v>1.2993542257184478</v>
       </c>
       <c r="E9">
         <f t="shared" si="2"/>
-        <v>0.291100989596631</v>
+        <v>0.29935422571844783</v>
       </c>
       <c r="F9">
         <f t="shared" si="3"/>
-        <v>1.096234787010939</v>
+        <v>1.1019953632217978</v>
       </c>
       <c r="G9">
         <f t="shared" si="4"/>
-        <v>0.2655462069310579</v>
+        <v>0.27164744581434053</v>
       </c>
       <c r="H9">
         <v>1700</v>
@@ -3021,29 +3021,29 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>0.74670204111011751</v>
+        <v>0.75857002059362821</v>
       </c>
       <c r="B10">
-        <v>102.079381</v>
+        <v>58.794444439999999</v>
       </c>
       <c r="C10">
-        <v>78.720592999999994</v>
+        <v>81.234813389999999</v>
       </c>
       <c r="D10">
         <f t="shared" si="1"/>
-        <v>1.2703156339282151</v>
+        <v>1.2309993194655384</v>
       </c>
       <c r="E10">
         <f t="shared" si="2"/>
-        <v>0.27031563392821512</v>
+        <v>0.23099931946553842</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>1.0671844144063189</v>
+        <v>0.95679633504306183</v>
       </c>
       <c r="G10">
         <f t="shared" si="4"/>
-        <v>0.25329795888988249</v>
+        <v>0.24142997940637179</v>
       </c>
       <c r="H10">
         <v>1800</v>
@@ -3052,29 +3052,29 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>0.76484099056244248</v>
+        <v>0.80896489060458188</v>
       </c>
       <c r="B11">
-        <v>104.559102</v>
+        <v>62.700396830000003</v>
       </c>
       <c r="C11">
-        <v>80.309307000000004</v>
+        <v>86.02606625</v>
       </c>
       <c r="D11">
         <f t="shared" si="1"/>
-        <v>1.2451856918650785</v>
+        <v>1.1624383673361329</v>
       </c>
       <c r="E11">
         <f t="shared" si="2"/>
-        <v>0.24518569186507855</v>
+        <v>0.16243836733613293</v>
       </c>
       <c r="F11">
         <f t="shared" si="3"/>
-        <v>1.0426378834113241</v>
+        <v>0.85030635389595521</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>0.23515900943755752</v>
+        <v>0.19103510939541812</v>
       </c>
       <c r="H11">
         <v>1900</v>
@@ -3083,29 +3083,29 @@
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>0.79032315687172672</v>
+        <v>0.82071498972899004</v>
       </c>
       <c r="B12">
-        <v>108.042692</v>
+        <v>63.611111110000003</v>
       </c>
       <c r="C12">
-        <v>81.890827999999999</v>
+        <v>85.754771739999995</v>
       </c>
       <c r="D12">
         <f t="shared" si="1"/>
-        <v>1.2211379765265045</v>
+        <v>1.1661158670352494</v>
       </c>
       <c r="E12">
         <f t="shared" si="2"/>
-        <v>0.22113797652650447</v>
+        <v>0.16611586703524939</v>
       </c>
       <c r="F12">
         <f t="shared" si="3"/>
-        <v>1.0546609402699736</v>
+        <v>0.92654632299792439</v>
       </c>
       <c r="G12">
         <f t="shared" si="4"/>
-        <v>0.20967684312827328</v>
+        <v>0.17928501027100996</v>
       </c>
       <c r="H12">
         <v>2000</v>
@@ -3114,29 +3114,29 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>0.81145060771586064</v>
+        <v>0.86115801599777275</v>
       </c>
       <c r="B13">
-        <v>110.93096199999999</v>
+        <v>66.745726500000004</v>
       </c>
       <c r="C13">
-        <v>76.480919</v>
+        <v>91.219768090000002</v>
       </c>
       <c r="D13">
         <f t="shared" si="1"/>
-        <v>1.3075156693658452</v>
+        <v>1.09625360921042</v>
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>0.30751566936584518</v>
+        <v>9.6253609210420032E-2</v>
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>1.630955505295008</v>
+        <v>0.69326011078087135</v>
       </c>
       <c r="G13">
         <f t="shared" si="4"/>
-        <v>0.18854939228413936</v>
+        <v>0.13884198400222725</v>
       </c>
       <c r="H13">
         <v>2100</v>
@@ -3145,29 +3145,29 @@
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>0.83968260435568121</v>
+        <v>0.86934586786814638</v>
       </c>
       <c r="B14">
-        <v>114.79047300000001</v>
+        <v>67.380341880000003</v>
       </c>
       <c r="C14">
-        <v>92.520120000000006</v>
+        <v>93.726887009999999</v>
       </c>
       <c r="D14">
         <f t="shared" si="1"/>
-        <v>1.0808459824738663</v>
+        <v>1.0669297059800003</v>
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>8.0845982473866318E-2</v>
+        <v>6.6929705980000254E-2</v>
       </c>
       <c r="F14">
         <f t="shared" si="3"/>
-        <v>0.50428702480441823</v>
+        <v>0.51226627805736824</v>
       </c>
       <c r="G14">
         <f t="shared" si="4"/>
-        <v>0.16031739564431879</v>
+        <v>0.13065413213185362</v>
       </c>
       <c r="H14">
         <v>2200</v>
@@ -3176,29 +3176,29 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>0.89092461116469701</v>
+        <v>0.9031302513052597</v>
       </c>
       <c r="B15">
-        <v>121.795613</v>
+        <v>69.998866210000003</v>
       </c>
       <c r="C15">
-        <v>83.858969000000002</v>
+        <v>96.663669780000006</v>
       </c>
       <c r="D15">
         <f t="shared" si="1"/>
-        <v>1.1924782905451652</v>
+        <v>1.0345148309348617</v>
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>0.19247829054516519</v>
+        <v>3.451483093486174E-2</v>
       </c>
       <c r="F15">
         <f t="shared" si="3"/>
-        <v>1.7646353829257979</v>
+        <v>0.35630143981921758</v>
       </c>
       <c r="G15">
         <f t="shared" si="4"/>
-        <v>0.10907538883530299</v>
+        <v>9.6869748694740299E-2</v>
       </c>
       <c r="H15">
         <v>2300</v>
@@ -3210,7 +3210,7 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>136.70697999999999</v>
+        <v>77.506944439999998</v>
       </c>
       <c r="C16">
         <v>100</v>

</xml_diff>

<commit_message>
Update rank-based performance workbook
</commit_message>
<xml_diff>
--- a/job_scheduler/data/all_model_data_by_rank.xlsx
+++ b/job_scheduler/data/all_model_data_by_rank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/imtiazevan/Desktop/Projects/temp/MPR_System_Beta/job_scheduler/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A479DE6-2FE6-A640-871F-73D0BC1CF9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0ABE18-9B8A-7D43-86C9-7F56BA5FE77F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="920" yWindow="500" windowWidth="28800" windowHeight="16300" activeTab="5" xr2:uid="{15444B7F-6FA5-5E4D-9AAE-4CEB8B7D2F02}"/>
+    <workbookView xWindow="-20" yWindow="500" windowWidth="28800" windowHeight="16300" activeTab="6" xr2:uid="{15444B7F-6FA5-5E4D-9AAE-4CEB8B7D2F02}"/>
   </bookViews>
   <sheets>
     <sheet name="minimd_rank2" sheetId="20" r:id="rId1"/>
@@ -4576,29 +4576,29 @@
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f t="shared" ref="A2:A15" si="0">B2/$B$16</f>
-        <v>0.5950119502599206</v>
+        <v>0.64264024292792366</v>
       </c>
       <c r="B2">
-        <v>74.243625665452498</v>
+        <v>93.511627906976699</v>
       </c>
       <c r="C2">
-        <v>59.396140458614688</v>
+        <v>57.838754853180617</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:D15" si="1">1/C2*100</f>
-        <v>1.6836110768792589</v>
+        <v>1.7289445503078786</v>
       </c>
       <c r="E2">
         <f t="shared" ref="E2:E15" si="2">D2-$D$16</f>
-        <v>0.68361107687925893</v>
+        <v>0.72894455030787864</v>
       </c>
       <c r="F2">
         <f>IFERROR(E2/G2,0)</f>
-        <v>1.687978391752545</v>
+        <v>2.0398059263311423</v>
       </c>
       <c r="G2">
         <f>$A$16-A2</f>
-        <v>0.4049880497400794</v>
+        <v>0.35735975707207634</v>
       </c>
       <c r="H2">
         <v>1000</v>
@@ -4607,29 +4607,29 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>0.60757316040128151</v>
+        <v>0.62202333386607289</v>
       </c>
       <c r="B3">
-        <v>75.810971973762605</v>
+        <v>90.511627906976699</v>
       </c>
       <c r="C3">
-        <v>62.821920806558076</v>
+        <v>61.359694645656369</v>
       </c>
       <c r="D3">
         <f t="shared" si="1"/>
-        <v>1.5918010579129067</v>
+        <v>1.6297343162720408</v>
       </c>
       <c r="E3">
         <f t="shared" si="2"/>
-        <v>0.59180105791290671</v>
+        <v>0.62973431627204079</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F16" si="3">IFERROR(E3/G3,0)</f>
-        <v>1.508054491171045</v>
+        <v>1.6660666456296784</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G16" si="4">$A$16-A3</f>
-        <v>0.39242683959871849</v>
+        <v>0.37797666613392711</v>
       </c>
       <c r="H3">
         <v>1100</v>
@@ -4638,29 +4638,29 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>0.65832603402222156</v>
+        <v>0.67012945501039145</v>
       </c>
       <c r="B4">
-        <v>82.143747893495103</v>
+        <v>97.511627906976699</v>
       </c>
       <c r="C4">
-        <v>69.583103746042326</v>
+        <v>68.07162974050388</v>
       </c>
       <c r="D4">
         <f t="shared" si="1"/>
-        <v>1.4371304902547941</v>
+        <v>1.4690407792675213</v>
       </c>
       <c r="E4">
         <f t="shared" si="2"/>
-        <v>0.43713049025479411</v>
+        <v>0.4690407792675213</v>
       </c>
       <c r="F4">
         <f t="shared" si="3"/>
-        <v>1.279378980496348</v>
+        <v>1.421893486374471</v>
       </c>
       <c r="G4">
         <f t="shared" si="4"/>
-        <v>0.34167396597777844</v>
+        <v>0.32987054498960855</v>
       </c>
       <c r="H4">
         <v>1200</v>
@@ -4669,29 +4669,29 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>0.67009163123171633</v>
+        <v>0.71823557615470535</v>
       </c>
       <c r="B5">
-        <v>83.611820248295103</v>
+        <v>104.511627906976</v>
       </c>
       <c r="C5">
-        <v>73.368990705428885</v>
+        <v>72.093335730372004</v>
       </c>
       <c r="D5">
         <f t="shared" si="1"/>
-        <v>1.3629736355716362</v>
+        <v>1.3870907620920538</v>
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>0.3629736355716362</v>
+        <v>0.38709076209205384</v>
       </c>
       <c r="F5">
         <f t="shared" si="3"/>
-        <v>1.1002256078765205</v>
+        <v>1.3738099253601639</v>
       </c>
       <c r="G5">
         <f t="shared" si="4"/>
-        <v>0.32990836876828367</v>
+        <v>0.28176442384529465</v>
       </c>
       <c r="H5">
         <v>1300</v>
@@ -4700,29 +4700,29 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>0.68574875314369688</v>
+        <v>0.73198018219593919</v>
       </c>
       <c r="B6">
-        <v>85.5654642006958</v>
+        <v>106.511627906976</v>
       </c>
       <c r="C6">
-        <v>77.268366171374709</v>
+        <v>75.273068283416706</v>
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>1.2941906883110281</v>
+        <v>1.3284963969248857</v>
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>0.29419068831102813</v>
+        <v>0.32849639692488575</v>
       </c>
       <c r="F6">
         <f t="shared" si="3"/>
-        <v>0.93616394924139146</v>
+        <v>1.2256421917465712</v>
       </c>
       <c r="G6">
         <f t="shared" si="4"/>
-        <v>0.31425124685630312</v>
+        <v>0.26801981780406081</v>
       </c>
       <c r="H6">
         <v>1400</v>
@@ -4731,29 +4731,29 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>0.7146061430356202</v>
+        <v>0.77321400031964083</v>
       </c>
       <c r="B7">
-        <v>89.166193987521197</v>
+        <v>112.511627906976</v>
       </c>
       <c r="C7">
-        <v>79.748018276212349</v>
+        <v>78.804841635776938</v>
       </c>
       <c r="D7">
         <f t="shared" si="1"/>
-        <v>1.2539496549449496</v>
+        <v>1.2689575656047076</v>
       </c>
       <c r="E7">
         <f t="shared" si="2"/>
-        <v>0.25394965494494959</v>
+        <v>0.26895756560470763</v>
       </c>
       <c r="F7">
         <f t="shared" si="3"/>
-        <v>0.88982172793104375</v>
+        <v>1.1859531275466151</v>
       </c>
       <c r="G7">
         <f t="shared" si="4"/>
-        <v>0.2853938569643798</v>
+        <v>0.22678599968035917</v>
       </c>
       <c r="H7">
         <v>1500</v>
@@ -4762,29 +4762,29 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>0.7524884511295965</v>
+        <v>0.80757551542272554</v>
       </c>
       <c r="B8">
-        <v>93.893023255813901</v>
+        <v>117.511627906976</v>
       </c>
       <c r="C8">
-        <v>83.475889289054123</v>
+        <v>81.274136815968063</v>
       </c>
       <c r="D8">
         <f t="shared" si="1"/>
-        <v>1.1979506999168035</v>
+        <v>1.2304037165775574</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>0.19795069991680347</v>
+        <v>0.23040371657755743</v>
       </c>
       <c r="F8">
         <f t="shared" si="3"/>
-        <v>0.79976348909864414</v>
+        <v>1.1973721383934961</v>
       </c>
       <c r="G8">
         <f t="shared" si="4"/>
-        <v>0.2475115488704035</v>
+        <v>0.19242448457727446</v>
       </c>
       <c r="H8">
         <v>1600</v>
@@ -4793,29 +4793,29 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>0.78687715674150316</v>
+        <v>0.8213201214639595</v>
       </c>
       <c r="B9">
-        <v>98.183932346722997</v>
+        <v>119.511627906976</v>
       </c>
       <c r="C9">
-        <v>86.015490523478405</v>
+        <v>83.922145186926457</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>1.1625812907816231</v>
+        <v>1.1915805986281935</v>
       </c>
       <c r="E9">
         <f t="shared" si="2"/>
-        <v>0.16258129078162309</v>
+        <v>0.19158059862819354</v>
       </c>
       <c r="F9">
         <f t="shared" si="3"/>
-        <v>0.76285248589907428</v>
+        <v>1.0722001839146702</v>
       </c>
       <c r="G9">
         <f t="shared" si="4"/>
-        <v>0.21312284325849684</v>
+        <v>0.1786798785360405</v>
       </c>
       <c r="H9">
         <v>1700</v>
@@ -4824,29 +4824,29 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>0.79208776380777435</v>
+        <v>0.86255393958766113</v>
       </c>
       <c r="B10">
-        <v>98.834094684385306</v>
+        <v>125.511627906976</v>
       </c>
       <c r="C10">
-        <v>87.116924468449824</v>
+        <v>87.038234352494626</v>
       </c>
       <c r="D10">
         <f t="shared" si="1"/>
-        <v>1.1478825797645773</v>
+        <v>1.1489203652157252</v>
       </c>
       <c r="E10">
         <f t="shared" si="2"/>
-        <v>0.1478825797645773</v>
+        <v>0.14892036521572516</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>0.71127405713558955</v>
+        <v>1.0834822385520786</v>
       </c>
       <c r="G10">
         <f t="shared" si="4"/>
-        <v>0.20791223619222565</v>
+        <v>0.13744606041233887</v>
       </c>
       <c r="H10">
         <v>1800</v>
@@ -4855,29 +4855,29 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>0.82570072092788871</v>
+        <v>0.86942624260827805</v>
       </c>
       <c r="B11">
-        <v>103.02820844099899</v>
+        <v>126.511627906976</v>
       </c>
       <c r="C11">
-        <v>89.95043133602401</v>
+        <v>88.470551593949025</v>
       </c>
       <c r="D11">
         <f t="shared" si="1"/>
-        <v>1.1117234071555948</v>
+        <v>1.1303196170740224</v>
       </c>
       <c r="E11">
         <f t="shared" si="2"/>
-        <v>0.11172340715559481</v>
+        <v>0.1303196170740224</v>
       </c>
       <c r="F11">
         <f t="shared" si="3"/>
-        <v>0.64098605427606203</v>
+        <v>0.99805366466603906</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>0.17429927907211129</v>
+        <v>0.13057375739172195</v>
       </c>
       <c r="H11">
         <v>1900</v>
@@ -4886,29 +4886,29 @@
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>0.85127463409273774</v>
+        <v>0.8831708486495119</v>
       </c>
       <c r="B12">
-        <v>106.21923684804599</v>
+        <v>128.511627906976</v>
       </c>
       <c r="C12">
-        <v>93.015448823007702</v>
+        <v>83.649183815415341</v>
       </c>
       <c r="D12">
         <f t="shared" si="1"/>
-        <v>1.0750902271114413</v>
+        <v>1.195468926758033</v>
       </c>
       <c r="E12">
         <f t="shared" si="2"/>
-        <v>7.509022711144131E-2</v>
+        <v>0.19546892675803296</v>
       </c>
       <c r="F12">
         <f t="shared" si="3"/>
-        <v>0.50489186329024627</v>
+        <v>1.6731177492818132</v>
       </c>
       <c r="G12">
         <f t="shared" si="4"/>
-        <v>0.14872536590726226</v>
+        <v>0.1168291513504881</v>
       </c>
       <c r="H12">
         <v>2000</v>
@@ -4917,29 +4917,29 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>0.87897460348064294</v>
+        <v>0.91753236375259672</v>
       </c>
       <c r="B13">
-        <v>109.675547527658</v>
+        <v>133.511627906976</v>
       </c>
       <c r="C13">
-        <v>94.3644608683108</v>
+        <v>89.797811431127656</v>
       </c>
       <c r="D13">
         <f t="shared" si="1"/>
-        <v>1.0597209911425638</v>
+        <v>1.1136128866202617</v>
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>5.9720991142563795E-2</v>
+        <v>0.1136128866202617</v>
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>0.49345833899426134</v>
+        <v>1.3776663402770819</v>
       </c>
       <c r="G13">
         <f t="shared" si="4"/>
-        <v>0.12102539651935706</v>
+        <v>8.2467636247403275E-2</v>
       </c>
       <c r="H13">
         <v>2100</v>
@@ -4948,29 +4948,29 @@
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>0.88962755766940005</v>
+        <v>0.93127696979383057</v>
       </c>
       <c r="B14">
-        <v>111.004787961696</v>
+        <v>135.511627906976</v>
       </c>
       <c r="C14">
-        <v>93.859791056327296</v>
+        <v>94.966583720516468</v>
       </c>
       <c r="D14">
         <f t="shared" si="1"/>
-        <v>1.065418949632946</v>
+        <v>1.0530019727180742</v>
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>6.5418949632946033E-2</v>
+        <v>5.3001972718074164E-2</v>
       </c>
       <c r="F14">
         <f t="shared" si="3"/>
-        <v>0.59271090003604199</v>
+        <v>0.77124033324881025</v>
       </c>
       <c r="G14">
         <f t="shared" si="4"/>
-        <v>0.11037244233059995</v>
+        <v>6.8723030206169433E-2</v>
       </c>
       <c r="H14">
         <v>2200</v>
@@ -4979,29 +4979,29 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>0.90542047643558499</v>
+        <v>0.95876618187629836</v>
       </c>
       <c r="B15">
-        <v>112.97537619699</v>
+        <v>139.511627906976</v>
       </c>
       <c r="C15">
-        <v>95.289944190919883</v>
+        <v>94.432698316945135</v>
       </c>
       <c r="D15">
         <f t="shared" si="1"/>
-        <v>1.0494286763317147</v>
+        <v>1.0589552324806952</v>
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>4.942867633171466E-2</v>
+        <v>5.895523248069523E-2</v>
       </c>
       <c r="F15">
         <f t="shared" si="3"/>
-        <v>0.52261498545243157</v>
+        <v>1.429778641983366</v>
       </c>
       <c r="G15">
         <f t="shared" si="4"/>
-        <v>9.4579523564415013E-2</v>
+        <v>4.1233818123701638E-2</v>
       </c>
       <c r="H15">
         <v>2300</v>
@@ -5013,7 +5013,7 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>124.77669672520101</v>
+        <v>145.511627906976</v>
       </c>
       <c r="C16">
         <v>100</v>

</xml_diff>